<commit_message>
fix ELS familly 7
</commit_message>
<xml_diff>
--- a/assets/prepared/CCI_02.xlsx
+++ b/assets/prepared/CCI_02.xlsx
@@ -52,22 +52,22 @@
     <t>_Z</t>
   </si>
   <si>
-    <t>K1</t>
-  </si>
-  <si>
-    <t>K2</t>
-  </si>
-  <si>
-    <t>K3</t>
-  </si>
-  <si>
-    <t>Overall Cost Index</t>
-  </si>
-  <si>
-    <t>Material Costs Index</t>
-  </si>
-  <si>
-    <t>Labour Costs Index</t>
+    <t>K0</t>
+  </si>
+  <si>
+    <t>K18</t>
+  </si>
+  <si>
+    <t>K19</t>
+  </si>
+  <si>
+    <t>Overall Index</t>
+  </si>
+  <si>
+    <t>Material Cost</t>
+  </si>
+  <si>
+    <t>Labour Cost</t>
   </si>
   <si>
     <t>2000-Q1</t>

</xml_diff>